<commit_message>
refactor(brand): rename FX·King → Rebound across the system
Full rebrand of the visible brand and internal naming:
- Display name FX·King → Rebound on landing, bot, miniapp, admin, docs.
- npm scope @fxking/* → @rebound/* (all package.json + imports + turbo
  filters in Dockerfile/CI).
- Infra names fxking-* → rebound-* (render.yaml), domains *.fxking.io/app
  → *.rebound.app (.env.example, vercel CSP, configs).
- Bot handle FxKingBot/FXKingBot → ReboundBot (+ /app deep link).
- Regenerated economics.xlsx + 4 legal .docx from rebranded generators.
- Tagline: "Every trade rebounds — in cash."

No behavioural change; compliance constants and gates untouched.

https://claude.ai/code/session_015A9R3NuW3DbezVMZHYA6VU
</commit_message>
<xml_diff>
--- a/docs/economics.xlsx
+++ b/docs/economics.xlsx
@@ -343,7 +343,7 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>FX·King</author>
+    <author>Rebound</author>
   </authors>
   <commentList>
     <comment ref="B5" authorId="0" shapeId="0">
@@ -726,7 +726,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>FX·KING — GAZDASÁGI MODELL</t>
+          <t>REBOUND — GAZDASÁGI MODELL</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>

</xml_diff>